<commit_message>
feat: Introduce Odoo mock data generation with sample Excel files and enhance the hydration guide to cover multi-line documents and product variant resolution.
</commit_message>
<xml_diff>
--- a/hydration/samples/1_contacts.xlsx
+++ b/hydration/samples/1_contacts.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,6 +451,21 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>street</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>parent_id/id</t>
         </is>
       </c>
@@ -476,7 +491,22 @@
           <t>info@acme.com</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>123 Industrial Way</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Metropolis</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -499,7 +529,10 @@
           <t>alice@acme.com</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
         <is>
           <t>comp_acme</t>
         </is>
@@ -526,7 +559,10 @@
           <t>bob@acme.com</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
         <is>
           <t>comp_acme</t>
         </is>
@@ -553,7 +589,22 @@
           <t>sales@betasupplies.com</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>456 Supplier Blvd</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Gotham</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>10002</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>